<commit_message>
x1499 more than one sample in a block (#625)
x1499: changing how blocks are represented

Previously info about a *block* was stored in a slot/sample link table
with an int for the highest section taken from the block. Block labware
was required to have exactly one slot and exactly one sample.
In the future we will support labware representing a block with
multiple samples in, where each sample may be spread across multiple
slots.
We represent that by marking a *sample* as a block by it having a
non-null blockHighestSection field. Labware can contain multiple
block-samples. Block-samples can be shared across multiple slots
in a piece of labware.

This commit has a small change to the graphql schema but other outward
facing behaviour should be largely unchanged.

x1404: support multiple samples in a block processing request

Block processing can take samples from multi-sample source labware
and can place multiple block-samples into destination labware.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/block_reg.xlsx
+++ b/src/test/resources/testdata/block_reg.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dr6/Code/stan/core/src/test/resources/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59177633-906C-AB42-8FD2-CE6F6D5BCB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1607B84-E4BC-FD4C-9C1F-7F427D261264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="760" windowWidth="27640" windowHeight="15900" activeTab="2" xr2:uid="{5C25E200-6C46-9D45-98E6-7DE84B4E9124}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
   <si>
     <t>DONOR INFO</t>
   </si>
@@ -190,6 +190,24 @@
   </si>
   <si>
     <t>Homo sapiens (Human)</t>
+  </si>
+  <si>
+    <t>Slot address</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>External barcode</t>
+  </si>
+  <si>
+    <t>XBC1</t>
+  </si>
+  <si>
+    <t>XBC2</t>
+  </si>
+  <si>
+    <t>XBC3</t>
   </si>
 </sst>
 </file>
@@ -559,7 +577,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E192D199-3D24-FD46-8181-D5EE66C2F681}">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -575,14 +593,16 @@
     <col min="11" max="11" width="33.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="41" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="41.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="59.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="31" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="33.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.1640625" customWidth="1"/>
+    <col min="15" max="15" width="59.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="59.5" customWidth="1"/>
+    <col min="17" max="17" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="33.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>0</v>
       </c>
@@ -592,11 +612,11 @@
       <c r="K1" t="s">
         <v>2</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -637,22 +657,28 @@
         <v>14</v>
       </c>
       <c r="N2" t="s">
+        <v>50</v>
+      </c>
+      <c r="O2" t="s">
         <v>15</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q2" t="s">
         <v>16</v>
       </c>
-      <c r="P2" t="s">
+      <c r="R2" t="s">
         <v>17</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="S2" t="s">
         <v>18</v>
       </c>
-      <c r="R2" t="s">
+      <c r="T2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -692,20 +718,26 @@
       <c r="M3">
         <v>1</v>
       </c>
-      <c r="N3">
+      <c r="N3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O3">
         <v>19</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q3" t="s">
         <v>27</v>
       </c>
-      <c r="P3" t="s">
+      <c r="R3" t="s">
         <v>28</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="S3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>35</v>
       </c>
@@ -739,20 +771,26 @@
       <c r="M4">
         <v>1</v>
       </c>
-      <c r="N4">
+      <c r="N4" t="s">
+        <v>51</v>
+      </c>
+      <c r="O4">
         <v>19</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q4" t="s">
         <v>27</v>
       </c>
-      <c r="P4" t="s">
+      <c r="R4" t="s">
         <v>28</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="S4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>36</v>
       </c>
@@ -789,19 +827,25 @@
       <c r="M5">
         <v>2</v>
       </c>
-      <c r="N5">
+      <c r="N5" t="s">
+        <v>51</v>
+      </c>
+      <c r="O5">
         <v>21</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q5" t="s">
         <v>27</v>
       </c>
-      <c r="P5" t="s">
+      <c r="R5" t="s">
         <v>41</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="S5" t="s">
         <v>39</v>
       </c>
-      <c r="R5" t="s">
+      <c r="T5" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>